<commit_message>
Adapt to TSAM v4.0
</commit_message>
<xml_diff>
--- a/test/data/expected_result_minisystem_segmentation.xlsx
+++ b/test/data/expected_result_minisystem_segmentation.xlsx
@@ -183,13 +183,13 @@
     <t>stateOfChargeOperationVariablesOptimum</t>
   </si>
   <si>
-    <t>LocationIn</t>
+    <t>locationIn</t>
   </si>
   <si>
     <t>Pipelines</t>
   </si>
   <si>
-    <t>LocationOut</t>
+    <t>locationOut</t>
   </si>
   <si>
     <t>periodsOrder</t>
@@ -205,16 +205,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -230,7 +222,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -238,30 +230,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -560,198 +534,182 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="E1" s="1" t="s">
+      <c r="D1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E1" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="1" t="s">
+      <c r="A2" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" t="s">
         <v>25</v>
       </c>
       <c r="D2">
-        <v>1520485.714285719</v>
+        <v>1708200.000000002</v>
       </c>
       <c r="E2">
         <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1" t="s">
+      <c r="B3" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" t="s">
         <v>26</v>
       </c>
       <c r="D3">
-        <v>1520485.714285718</v>
+        <v>1708200</v>
       </c>
       <c r="E3">
         <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="1"/>
-      <c r="B4" s="1" t="s">
+      <c r="B4" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="1"/>
-      <c r="B5" s="1" t="s">
+      <c r="B5" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="1"/>
-      <c r="B6" s="1" t="s">
+      <c r="B6" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="1"/>
-      <c r="B7" s="1" t="s">
+      <c r="B7" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="C7" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="1"/>
-      <c r="B8" s="1" t="s">
+      <c r="B8" t="s">
         <v>13</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="C8" t="s">
         <v>26</v>
       </c>
       <c r="D8">
-        <v>1895914.285714289</v>
+        <v>1895914.285714286</v>
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="1"/>
-      <c r="B9" s="1" t="s">
+      <c r="B9" t="s">
         <v>14</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="C9" t="s">
         <v>26</v>
       </c>
       <c r="D9">
-        <v>375428.571428571</v>
+        <v>187714.2857142857</v>
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="1"/>
-      <c r="B10" s="1" t="s">
+      <c r="B10" t="s">
         <v>15</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="C10" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="1"/>
-      <c r="B11" s="1" t="s">
+      <c r="B11" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="C11" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="1"/>
-      <c r="B12" s="1" t="s">
+      <c r="B12" t="s">
         <v>17</v>
       </c>
-      <c r="C12" s="1" t="s">
+      <c r="C12" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="1"/>
-      <c r="B13" s="1" t="s">
+      <c r="B13" t="s">
         <v>18</v>
       </c>
-      <c r="C13" s="1" t="s">
+      <c r="C13" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="1"/>
-      <c r="B14" s="1" t="s">
+      <c r="B14" t="s">
         <v>19</v>
       </c>
-      <c r="C14" s="1" t="s">
+      <c r="C14" t="s">
         <v>29</v>
       </c>
       <c r="D14">
-        <v>75085714.2857143</v>
+        <v>75085714.28571428</v>
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="1"/>
-      <c r="B15" s="1" t="s">
+      <c r="B15" t="s">
         <v>20</v>
       </c>
-      <c r="C15" s="1" t="s">
+      <c r="C15" t="s">
         <v>30</v>
       </c>
       <c r="D15">
-        <v>75085714.2857143</v>
+        <v>75085714.28571428</v>
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="1"/>
-      <c r="B16" s="1" t="s">
+      <c r="B16" t="s">
         <v>21</v>
       </c>
-      <c r="C16" s="1" t="s">
+      <c r="C16" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="1"/>
-      <c r="B17" s="1" t="s">
+      <c r="B17" t="s">
         <v>22</v>
       </c>
-      <c r="C17" s="1" t="s">
+      <c r="C17" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="1"/>
-      <c r="B18" s="1" t="s">
+      <c r="B18" t="s">
         <v>23</v>
       </c>
-      <c r="C18" s="1" t="s">
+      <c r="C18" t="s">
         <v>26</v>
       </c>
       <c r="D18">
@@ -759,22 +717,21 @@
       </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="1"/>
-      <c r="B19" s="1" t="s">
+      <c r="B19" t="s">
         <v>24</v>
       </c>
-      <c r="C19" s="1" t="s">
+      <c r="C19" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="1" t="s">
+      <c r="A20" t="s">
         <v>6</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="B20" t="s">
         <v>7</v>
       </c>
-      <c r="C20" s="1" t="s">
+      <c r="C20" t="s">
         <v>25</v>
       </c>
       <c r="D20">
@@ -785,11 +742,10 @@
       </c>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="1"/>
-      <c r="B21" s="1" t="s">
+      <c r="B21" t="s">
         <v>8</v>
       </c>
-      <c r="C21" s="1" t="s">
+      <c r="C21" t="s">
         <v>26</v>
       </c>
       <c r="D21">
@@ -800,47 +756,42 @@
       </c>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="1"/>
-      <c r="B22" s="1" t="s">
+      <c r="B22" t="s">
         <v>9</v>
       </c>
-      <c r="C22" s="1" t="s">
+      <c r="C22" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="23" spans="1:5">
-      <c r="A23" s="1"/>
-      <c r="B23" s="1" t="s">
+      <c r="B23" t="s">
         <v>10</v>
       </c>
-      <c r="C23" s="1" t="s">
+      <c r="C23" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="24" spans="1:5">
-      <c r="A24" s="1"/>
-      <c r="B24" s="1" t="s">
+      <c r="B24" t="s">
         <v>11</v>
       </c>
-      <c r="C24" s="1" t="s">
+      <c r="C24" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="25" spans="1:5">
-      <c r="A25" s="1"/>
-      <c r="B25" s="1" t="s">
+      <c r="B25" t="s">
         <v>12</v>
       </c>
-      <c r="C25" s="1" t="s">
+      <c r="C25" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="1"/>
-      <c r="B26" s="1" t="s">
+      <c r="B26" t="s">
         <v>13</v>
       </c>
-      <c r="C26" s="1" t="s">
+      <c r="C26" t="s">
         <v>26</v>
       </c>
       <c r="E26">
@@ -848,11 +799,10 @@
       </c>
     </row>
     <row r="27" spans="1:5">
-      <c r="A27" s="1"/>
-      <c r="B27" s="1" t="s">
+      <c r="B27" t="s">
         <v>14</v>
       </c>
-      <c r="C27" s="1" t="s">
+      <c r="C27" t="s">
         <v>26</v>
       </c>
       <c r="E27">
@@ -860,101 +810,91 @@
       </c>
     </row>
     <row r="28" spans="1:5">
-      <c r="A28" s="1"/>
-      <c r="B28" s="1" t="s">
+      <c r="B28" t="s">
         <v>15</v>
       </c>
-      <c r="C28" s="1" t="s">
+      <c r="C28" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="29" spans="1:5">
-      <c r="A29" s="1"/>
-      <c r="B29" s="1" t="s">
+      <c r="B29" t="s">
         <v>16</v>
       </c>
-      <c r="C29" s="1" t="s">
+      <c r="C29" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="30" spans="1:5">
-      <c r="A30" s="1"/>
-      <c r="B30" s="1" t="s">
+      <c r="B30" t="s">
         <v>17</v>
       </c>
-      <c r="C30" s="1" t="s">
+      <c r="C30" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="31" spans="1:5">
-      <c r="A31" s="1"/>
-      <c r="B31" s="1" t="s">
+      <c r="B31" t="s">
         <v>18</v>
       </c>
-      <c r="C31" s="1" t="s">
+      <c r="C31" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="32" spans="1:5">
-      <c r="A32" s="1"/>
-      <c r="B32" s="1" t="s">
+      <c r="B32" t="s">
         <v>19</v>
       </c>
-      <c r="C32" s="1" t="s">
+      <c r="C32" t="s">
         <v>32</v>
       </c>
       <c r="E32">
         <v>52560000</v>
       </c>
     </row>
-    <row r="33" spans="1:5">
-      <c r="A33" s="1"/>
-      <c r="B33" s="1" t="s">
+    <row r="33" spans="2:5">
+      <c r="B33" t="s">
         <v>20</v>
       </c>
-      <c r="C33" s="1" t="s">
+      <c r="C33" t="s">
         <v>33</v>
       </c>
       <c r="E33">
         <v>52560000</v>
       </c>
     </row>
-    <row r="34" spans="1:5">
-      <c r="A34" s="1"/>
-      <c r="B34" s="1" t="s">
+    <row r="34" spans="2:5">
+      <c r="B34" t="s">
         <v>21</v>
       </c>
-      <c r="C34" s="1" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5">
-      <c r="A35" s="1"/>
-      <c r="B35" s="1" t="s">
+      <c r="C34" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="35" spans="2:5">
+      <c r="B35" t="s">
         <v>22</v>
       </c>
-      <c r="C35" s="1" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5">
-      <c r="A36" s="1"/>
-      <c r="B36" s="1" t="s">
+      <c r="C35" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="36" spans="2:5">
+      <c r="B36" t="s">
         <v>23</v>
       </c>
-      <c r="C36" s="1" t="s">
+      <c r="C36" t="s">
         <v>26</v>
       </c>
       <c r="E36">
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:5">
-      <c r="A37" s="1"/>
-      <c r="B37" s="1" t="s">
+    <row r="37" spans="2:5">
+      <c r="B37" t="s">
         <v>24</v>
       </c>
-      <c r="C37" s="1" t="s">
+      <c r="C37" t="s">
         <v>25</v>
       </c>
     </row>
@@ -973,42 +913,42 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>34</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>52</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>54</v>
       </c>
-      <c r="E1" s="1">
-        <v>0</v>
-      </c>
-      <c r="F1" s="1">
-        <v>1</v>
-      </c>
-      <c r="G1" s="1">
+      <c r="E1">
+        <v>0</v>
+      </c>
+      <c r="F1">
+        <v>1</v>
+      </c>
+      <c r="G1">
         <v>2</v>
       </c>
-      <c r="H1" s="1">
+      <c r="H1">
         <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:8">
-      <c r="A2" s="1" t="s">
+      <c r="A2" t="s">
         <v>36</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" t="s">
         <v>53</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D2" s="1" t="s">
+      <c r="C2" t="s">
+        <v>0</v>
+      </c>
+      <c r="D2" t="s">
         <v>1</v>
       </c>
       <c r="E2">
@@ -1025,25 +965,23 @@
       </c>
     </row>
     <row r="3" spans="1:8">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D3" s="1" t="s">
+      <c r="C3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D3" t="s">
         <v>0</v>
       </c>
       <c r="E3">
-        <v>1.50896230640301E-09</v>
+        <v>0</v>
       </c>
       <c r="F3">
         <v>0</v>
       </c>
       <c r="G3">
-        <v>1.50896230640301E-09</v>
+        <v>0</v>
       </c>
       <c r="H3">
-        <v>1.50896230640301E-09</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1061,30 +999,30 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>35</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="E1" s="1" t="s">
+      <c r="D1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E1" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="1" t="s">
+      <c r="A2" t="s">
         <v>39</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" t="s">
         <v>53</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" t="s">
         <v>0</v>
       </c>
       <c r="E2">
@@ -1092,9 +1030,7 @@
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1" t="s">
+      <c r="C3" t="s">
         <v>1</v>
       </c>
       <c r="D3">
@@ -1102,13 +1038,13 @@
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="1" t="s">
+      <c r="A4" t="s">
         <v>40</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" t="s">
         <v>53</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" t="s">
         <v>0</v>
       </c>
       <c r="E4">
@@ -1116,9 +1052,7 @@
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="1"/>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1" t="s">
+      <c r="C5" t="s">
         <v>1</v>
       </c>
       <c r="D5">
@@ -1126,13 +1060,13 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="1" t="s">
+      <c r="A6" t="s">
         <v>41</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" t="s">
         <v>53</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" t="s">
         <v>0</v>
       </c>
       <c r="E6">
@@ -1140,9 +1074,7 @@
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="1"/>
-      <c r="B7" s="1"/>
-      <c r="C7" s="1" t="s">
+      <c r="C7" t="s">
         <v>1</v>
       </c>
       <c r="D7">
@@ -1168,15 +1100,15 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="B1" s="1">
-        <v>0</v>
-      </c>
-      <c r="C1" s="1">
+      <c r="B1">
+        <v>0</v>
+      </c>
+      <c r="C1">
         <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:3">
-      <c r="A2" s="1" t="s">
+      <c r="A2" t="s">
         <v>55</v>
       </c>
       <c r="B2">
@@ -1187,18 +1119,18 @@
       </c>
     </row>
     <row r="4" spans="1:3">
-      <c r="A4" s="1" t="s">
+      <c r="A4" t="s">
         <v>57</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" t="s">
         <v>56</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="5" spans="1:3">
-      <c r="A5" s="1">
+      <c r="A5">
         <v>0</v>
       </c>
       <c r="B5">
@@ -1209,7 +1141,7 @@
       </c>
     </row>
     <row r="6" spans="1:3">
-      <c r="A6" s="1">
+      <c r="A6">
         <v>1</v>
       </c>
       <c r="B6">
@@ -1230,57 +1162,56 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>34</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>35</v>
       </c>
-      <c r="D1" s="1">
-        <v>0</v>
-      </c>
-      <c r="E1" s="1">
-        <v>1</v>
-      </c>
-      <c r="F1" s="1">
+      <c r="D1">
+        <v>0</v>
+      </c>
+      <c r="E1">
+        <v>1</v>
+      </c>
+      <c r="F1">
         <v>2</v>
       </c>
-      <c r="G1" s="1">
+      <c r="G1">
         <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:7">
-      <c r="A2" s="1" t="s">
+      <c r="A2" t="s">
         <v>36</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" t="s">
         <v>0</v>
       </c>
       <c r="D2">
-        <v>18771428.5714286</v>
+        <v>37542857.14285714</v>
       </c>
       <c r="E2">
-        <v>37542857.1428571</v>
+        <v>18771428.57142857</v>
       </c>
       <c r="F2">
-        <v>0</v>
+        <v>18771428.57142857</v>
       </c>
       <c r="G2">
-        <v>18771428.5714286</v>
+        <v>-0</v>
       </c>
     </row>
     <row r="3" spans="1:7">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1" t="s">
+      <c r="B3" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" t="s">
         <v>1</v>
       </c>
       <c r="D3">
@@ -1310,114 +1241,108 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="E1" s="1" t="s">
+      <c r="D1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E1" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="1" t="s">
+      <c r="A2" t="s">
         <v>37</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" t="s">
         <v>25</v>
       </c>
       <c r="D2">
-        <v>1491681.331689215</v>
+        <v>1491681.331689218</v>
       </c>
       <c r="E2">
         <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1" t="s">
+      <c r="B3" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" t="s">
         <v>26</v>
       </c>
       <c r="D3">
-        <v>1491681.331689214</v>
+        <v>1491681.331689217</v>
       </c>
       <c r="E3">
         <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="1"/>
-      <c r="B4" s="1" t="s">
+      <c r="B4" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" t="s">
         <v>27</v>
       </c>
       <c r="D4">
-        <v>17142.8571428571</v>
+        <v>17142.85714285714</v>
       </c>
       <c r="E4">
         <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="1"/>
-      <c r="B5" s="1" t="s">
+      <c r="B5" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" t="s">
         <v>26</v>
       </c>
       <c r="D5">
-        <v>1277395.6174035</v>
+        <v>1277395.617403503</v>
       </c>
       <c r="E5">
         <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="1"/>
-      <c r="B6" s="1" t="s">
+      <c r="B6" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="1"/>
-      <c r="B7" s="1" t="s">
+      <c r="B7" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="C7" t="s">
         <v>27</v>
       </c>
       <c r="D7">
-        <v>17142.8571428571</v>
+        <v>17142.85714285714</v>
       </c>
       <c r="E7">
         <v>-0</v>
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="1"/>
-      <c r="B8" s="1" t="s">
+      <c r="B8" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="C8" t="s">
         <v>27</v>
       </c>
       <c r="D8">
@@ -1428,26 +1353,24 @@
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="1"/>
-      <c r="B9" s="1" t="s">
+      <c r="B9" t="s">
         <v>16</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="C9" t="s">
         <v>25</v>
       </c>
       <c r="D9">
-        <v>8571428.57142855</v>
+        <v>8571428.571428571</v>
       </c>
       <c r="E9">
         <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="1"/>
-      <c r="B10" s="1" t="s">
+      <c r="B10" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="C10" t="s">
         <v>25</v>
       </c>
       <c r="D10">
@@ -1458,74 +1381,68 @@
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="1"/>
-      <c r="B11" s="1" t="s">
+      <c r="B11" t="s">
         <v>18</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="C11" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="1"/>
-      <c r="B12" s="1" t="s">
+      <c r="B12" t="s">
         <v>19</v>
       </c>
-      <c r="C12" s="1" t="s">
+      <c r="C12" t="s">
         <v>29</v>
       </c>
       <c r="D12">
-        <v>75085714.2857143</v>
+        <v>75085714.28571428</v>
       </c>
       <c r="E12">
         <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="1"/>
-      <c r="B13" s="1" t="s">
+      <c r="B13" t="s">
         <v>20</v>
       </c>
-      <c r="C13" s="1" t="s">
+      <c r="C13" t="s">
         <v>30</v>
       </c>
       <c r="D13">
-        <v>75085714.2857143</v>
+        <v>75085714.28571428</v>
       </c>
       <c r="E13">
         <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="1"/>
-      <c r="B14" s="1" t="s">
+      <c r="B14" t="s">
         <v>21</v>
       </c>
-      <c r="C14" s="1" t="s">
+      <c r="C14" t="s">
         <v>26</v>
       </c>
       <c r="D14">
-        <v>214285.7142857138</v>
+        <v>214285.7142857143</v>
       </c>
       <c r="E14">
         <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="1"/>
-      <c r="B15" s="1" t="s">
+      <c r="B15" t="s">
         <v>22</v>
       </c>
-      <c r="C15" s="1" t="s">
+      <c r="C15" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="1"/>
-      <c r="B16" s="1" t="s">
+      <c r="B16" t="s">
         <v>23</v>
       </c>
-      <c r="C16" s="1" t="s">
+      <c r="C16" t="s">
         <v>26</v>
       </c>
       <c r="D16">
@@ -1535,12 +1452,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:5">
-      <c r="A17" s="1"/>
-      <c r="B17" s="1" t="s">
+    <row r="17" spans="2:5">
+      <c r="B17" t="s">
         <v>24</v>
       </c>
-      <c r="C17" s="1" t="s">
+      <c r="C17" t="s">
         <v>25</v>
       </c>
       <c r="D17">
@@ -1564,68 +1480,66 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>34</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>35</v>
       </c>
-      <c r="D1" s="1">
-        <v>0</v>
-      </c>
-      <c r="E1" s="1">
-        <v>1</v>
-      </c>
-      <c r="F1" s="1">
+      <c r="D1">
+        <v>0</v>
+      </c>
+      <c r="E1">
+        <v>1</v>
+      </c>
+      <c r="F1">
         <v>2</v>
       </c>
-      <c r="G1" s="1">
+      <c r="G1">
         <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:7">
-      <c r="A2" s="1" t="s">
+      <c r="A2" t="s">
         <v>36</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" t="s">
         <v>37</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" t="s">
         <v>0</v>
       </c>
       <c r="D2">
-        <v>18771428.5714286</v>
+        <v>37542857.14285714</v>
       </c>
       <c r="E2">
-        <v>37542857.1428571</v>
+        <v>18771428.57142857</v>
       </c>
       <c r="F2">
-        <v>0</v>
+        <v>18771428.57142857</v>
       </c>
       <c r="G2">
-        <v>18771428.5714286</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:7">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1" t="s">
+      <c r="C3" t="s">
         <v>1</v>
       </c>
       <c r="D3">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="F3">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="G3">
-        <v>0</v>
+        <v>-0</v>
       </c>
     </row>
   </sheetData>
@@ -1643,52 +1557,52 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1" s="1" t="s">
+      <c r="C1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:4">
-      <c r="A2" s="1" t="s">
+      <c r="A2" t="s">
         <v>39</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" t="s">
         <v>37</v>
       </c>
       <c r="C2">
-        <v>17142.8571428571</v>
+        <v>17142.85714285714</v>
       </c>
       <c r="D2">
         <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:4">
-      <c r="A3" s="1" t="s">
+      <c r="A3" t="s">
         <v>40</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" t="s">
         <v>37</v>
       </c>
       <c r="C3">
-        <v>17142.8571428571</v>
+        <v>17142.85714285714</v>
       </c>
       <c r="D3">
         <v>-0</v>
       </c>
     </row>
     <row r="4" spans="1:4">
-      <c r="A4" s="1" t="s">
+      <c r="A4" t="s">
         <v>41</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" t="s">
         <v>37</v>
       </c>
       <c r="C4">
@@ -1709,114 +1623,108 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="E1" s="1" t="s">
+      <c r="D1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E1" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="1" t="s">
+      <c r="A2" t="s">
         <v>42</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" t="s">
         <v>25</v>
       </c>
       <c r="D2">
-        <v>871039.1602304186</v>
+        <v>871039.1602304169</v>
       </c>
       <c r="E2">
-        <v>1.000277975790437E-10</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1" t="s">
+      <c r="B3" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" t="s">
         <v>26</v>
       </c>
       <c r="D3">
-        <v>871039.1602304177</v>
+        <v>871039.1602304161</v>
       </c>
       <c r="E3">
-        <v>1.000277975790436E-10</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="1"/>
-      <c r="B4" s="1" t="s">
+      <c r="B4" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" t="s">
         <v>32</v>
       </c>
       <c r="D4">
-        <v>19611940.2985075</v>
+        <v>19611940.29850746</v>
       </c>
       <c r="E4">
-        <v>2.25218254687017E-09</v>
+        <v>-0</v>
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="1"/>
-      <c r="B5" s="1" t="s">
+      <c r="B5" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" t="s">
         <v>26</v>
       </c>
       <c r="D5">
-        <v>871039.1602304177</v>
+        <v>871039.1602304161</v>
       </c>
       <c r="E5">
-        <v>1.000277975790436E-10</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="1"/>
-      <c r="B6" s="1" t="s">
+      <c r="B6" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="1"/>
-      <c r="B7" s="1" t="s">
+      <c r="B7" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="C7" t="s">
         <v>32</v>
       </c>
       <c r="D7">
-        <v>19611940.2985075</v>
+        <v>19611940.29850746</v>
       </c>
       <c r="E7">
-        <v>2.25218254687017E-09</v>
+        <v>-0</v>
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="1"/>
-      <c r="B8" s="1" t="s">
+      <c r="B8" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="C8" t="s">
         <v>32</v>
       </c>
       <c r="D8">
@@ -1827,26 +1735,24 @@
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="1"/>
-      <c r="B9" s="1" t="s">
+      <c r="B9" t="s">
         <v>16</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="C9" t="s">
         <v>25</v>
       </c>
       <c r="D9">
-        <v>9805970.14925375</v>
+        <v>9805970.149253732</v>
       </c>
       <c r="E9">
-        <v>1.126091273435085E-09</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="1"/>
-      <c r="B10" s="1" t="s">
+      <c r="B10" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="C10" t="s">
         <v>25</v>
       </c>
       <c r="D10">
@@ -1857,80 +1763,74 @@
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="1"/>
-      <c r="B11" s="1" t="s">
+      <c r="B11" t="s">
         <v>18</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="C11" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="1"/>
-      <c r="B12" s="1" t="s">
+      <c r="B12" t="s">
         <v>43</v>
       </c>
-      <c r="C12" s="1" t="s">
+      <c r="C12" t="s">
         <v>32</v>
       </c>
       <c r="D12">
         <v>13140000</v>
       </c>
       <c r="E12">
-        <v>1.50896230640301E-09</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="1"/>
-      <c r="B13" s="1" t="s">
+      <c r="B13" t="s">
         <v>44</v>
       </c>
-      <c r="C13" s="1" t="s">
+      <c r="C13" t="s">
         <v>33</v>
       </c>
       <c r="D13">
         <v>13140000</v>
       </c>
       <c r="E13">
-        <v>1.50896230640301E-09</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="1"/>
-      <c r="B14" s="1" t="s">
+      <c r="B14" t="s">
         <v>45</v>
       </c>
-      <c r="C14" s="1" t="s">
+      <c r="C14" t="s">
         <v>32</v>
       </c>
       <c r="D14">
         <v>13140000</v>
       </c>
       <c r="E14">
-        <v>1.50896230640301E-09</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="1"/>
-      <c r="B15" s="1" t="s">
+      <c r="B15" t="s">
         <v>46</v>
       </c>
-      <c r="C15" s="1" t="s">
+      <c r="C15" t="s">
         <v>33</v>
       </c>
       <c r="D15">
         <v>13140000</v>
       </c>
       <c r="E15">
-        <v>1.50896230640301E-09</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="1"/>
-      <c r="B16" s="1" t="s">
+      <c r="B16" t="s">
         <v>21</v>
       </c>
-      <c r="C16" s="1" t="s">
+      <c r="C16" t="s">
         <v>26</v>
       </c>
       <c r="D16">
@@ -1940,12 +1840,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:5">
-      <c r="A17" s="1"/>
-      <c r="B17" s="1" t="s">
+    <row r="17" spans="2:5">
+      <c r="B17" t="s">
         <v>47</v>
       </c>
-      <c r="C17" s="1" t="s">
+      <c r="C17" t="s">
         <v>26</v>
       </c>
       <c r="D17">
@@ -1955,12 +1854,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:5">
-      <c r="A18" s="1"/>
-      <c r="B18" s="1" t="s">
+    <row r="18" spans="2:5">
+      <c r="B18" t="s">
         <v>48</v>
       </c>
-      <c r="C18" s="1" t="s">
+      <c r="C18" t="s">
         <v>26</v>
       </c>
       <c r="D18">
@@ -1970,21 +1868,19 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:5">
-      <c r="A19" s="1"/>
-      <c r="B19" s="1" t="s">
+    <row r="19" spans="2:5">
+      <c r="B19" t="s">
         <v>22</v>
       </c>
-      <c r="C19" s="1" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5">
-      <c r="A20" s="1"/>
-      <c r="B20" s="1" t="s">
+      <c r="C19" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="20" spans="2:5">
+      <c r="B20" t="s">
         <v>24</v>
       </c>
-      <c r="C20" s="1" t="s">
+      <c r="C20" t="s">
         <v>25</v>
       </c>
       <c r="D20">
@@ -2008,152 +1904,146 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>34</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>35</v>
       </c>
-      <c r="D1" s="1">
-        <v>0</v>
-      </c>
-      <c r="E1" s="1">
-        <v>1</v>
-      </c>
-      <c r="F1" s="1">
+      <c r="D1">
+        <v>0</v>
+      </c>
+      <c r="E1">
+        <v>1</v>
+      </c>
+      <c r="F1">
         <v>2</v>
       </c>
-      <c r="G1" s="1">
+      <c r="G1">
         <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:7">
-      <c r="A2" s="1" t="s">
+      <c r="A2" t="s">
         <v>49</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" t="s">
         <v>42</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" t="s">
         <v>0</v>
       </c>
       <c r="D2">
-        <v>0</v>
+        <v>13140000</v>
       </c>
       <c r="E2">
+        <v>0</v>
+      </c>
+      <c r="F2">
+        <v>-0</v>
+      </c>
+      <c r="G2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
+      <c r="C3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>-0</v>
+      </c>
+      <c r="E3">
+        <v>0</v>
+      </c>
+      <c r="F3">
+        <v>-0</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B4" t="s">
+        <v>42</v>
+      </c>
+      <c r="C4" t="s">
+        <v>0</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>-0</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4">
         <v>13140000</v>
       </c>
-      <c r="F2">
-        <v>0</v>
-      </c>
-      <c r="G2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D3">
-        <v>0</v>
-      </c>
-      <c r="E3">
-        <v>1.50896230640301E-09</v>
-      </c>
-      <c r="F3">
-        <v>0</v>
-      </c>
-      <c r="G3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7">
-      <c r="A4" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="B4" s="1" t="s">
+    </row>
+    <row r="5" spans="1:7">
+      <c r="C5" t="s">
+        <v>1</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5">
+        <v>-0</v>
+      </c>
+      <c r="F5">
+        <v>0</v>
+      </c>
+      <c r="G5">
+        <v>-0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B6" t="s">
         <v>42</v>
       </c>
-      <c r="C4" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D4">
-        <v>0</v>
-      </c>
-      <c r="E4">
-        <v>0</v>
-      </c>
-      <c r="F4">
-        <v>13140000</v>
-      </c>
-      <c r="G4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7">
-      <c r="A5" s="1"/>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D5">
-        <v>0</v>
-      </c>
-      <c r="E5">
-        <v>0</v>
-      </c>
-      <c r="F5">
-        <v>1.50896230640301E-09</v>
-      </c>
-      <c r="G5">
-        <v>5.13302352179869E-25</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7">
-      <c r="A6" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" t="s">
         <v>0</v>
       </c>
       <c r="D6">
-        <v>6471940.29850747</v>
+        <v>6471940.298507463</v>
       </c>
       <c r="E6">
-        <v>6471940.29850747</v>
+        <v>19611940.29850746</v>
       </c>
       <c r="F6">
-        <v>19611940.2985075</v>
+        <v>19611940.29850746</v>
       </c>
       <c r="G6">
-        <v>6471940.2985075</v>
+        <v>19611940.29850746</v>
       </c>
     </row>
     <row r="7" spans="1:7">
-      <c r="A7" s="1"/>
-      <c r="B7" s="1"/>
-      <c r="C7" s="1" t="s">
+      <c r="C7" t="s">
         <v>1</v>
       </c>
       <c r="D7">
-        <v>7.43220240467156E-10</v>
+        <v>0</v>
       </c>
       <c r="E7">
-        <v>7.43220240467156E-10</v>
+        <v>-0</v>
       </c>
       <c r="F7">
-        <v>2.25218254687017E-09</v>
+        <v>0</v>
       </c>
       <c r="G7">
-        <v>7.432202404671603E-10</v>
+        <v>-0</v>
       </c>
     </row>
   </sheetData>
@@ -2175,59 +2065,59 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1" s="1" t="s">
+      <c r="C1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:4">
-      <c r="A2" s="1" t="s">
+      <c r="A2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C2">
+        <v>19611940.29850746</v>
+      </c>
+      <c r="D2">
+        <v>-0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" t="s">
         <v>40</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B3" t="s">
         <v>42</v>
       </c>
-      <c r="C2">
-        <v>19611940.2985075</v>
-      </c>
-      <c r="D2">
-        <v>2.25218254687017E-09</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4">
-      <c r="A3" s="1" t="s">
+      <c r="C3">
+        <v>19611940.29850746</v>
+      </c>
+      <c r="D3">
+        <v>-0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" t="s">
         <v>41</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B4" t="s">
         <v>42</v>
       </c>
-      <c r="C3">
-        <v>0</v>
-      </c>
-      <c r="D3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4">
-      <c r="A4" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>42</v>
-      </c>
       <c r="C4">
-        <v>19611940.2985075</v>
+        <v>0</v>
       </c>
       <c r="D4">
-        <v>2.25218254687017E-09</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -2241,36 +2131,36 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>52</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="F1" s="1" t="s">
+      <c r="E1" t="s">
+        <v>0</v>
+      </c>
+      <c r="F1" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:6">
-      <c r="A2" s="1" t="s">
+      <c r="A2" t="s">
         <v>53</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" t="s">
         <v>25</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" t="s">
         <v>0</v>
       </c>
       <c r="E2">
@@ -2281,10 +2171,7 @@
       </c>
     </row>
     <row r="3" spans="1:6">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1" t="s">
+      <c r="D3" t="s">
         <v>1</v>
       </c>
       <c r="E3">
@@ -2295,14 +2182,13 @@
       </c>
     </row>
     <row r="4" spans="1:6">
-      <c r="A4" s="1"/>
-      <c r="B4" s="1" t="s">
+      <c r="B4" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D4" s="1" t="s">
+      <c r="C4" t="s">
+        <v>26</v>
+      </c>
+      <c r="D4" t="s">
         <v>0</v>
       </c>
       <c r="E4">
@@ -2313,10 +2199,7 @@
       </c>
     </row>
     <row r="5" spans="1:6">
-      <c r="A5" s="1"/>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1" t="s">
+      <c r="D5" t="s">
         <v>1</v>
       </c>
       <c r="E5">
@@ -2327,14 +2210,13 @@
       </c>
     </row>
     <row r="6" spans="1:6">
-      <c r="A6" s="1"/>
-      <c r="B6" s="1" t="s">
+      <c r="B6" t="s">
         <v>9</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" t="s">
         <v>31</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="D6" t="s">
         <v>0</v>
       </c>
       <c r="F6">
@@ -2342,10 +2224,7 @@
       </c>
     </row>
     <row r="7" spans="1:6">
-      <c r="A7" s="1"/>
-      <c r="B7" s="1"/>
-      <c r="C7" s="1"/>
-      <c r="D7" s="1" t="s">
+      <c r="D7" t="s">
         <v>1</v>
       </c>
       <c r="E7">
@@ -2353,14 +2232,13 @@
       </c>
     </row>
     <row r="8" spans="1:6">
-      <c r="A8" s="1"/>
-      <c r="B8" s="1" t="s">
+      <c r="B8" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D8" s="1" t="s">
+      <c r="C8" t="s">
+        <v>26</v>
+      </c>
+      <c r="D8" t="s">
         <v>0</v>
       </c>
       <c r="F8">
@@ -2368,10 +2246,7 @@
       </c>
     </row>
     <row r="9" spans="1:6">
-      <c r="A9" s="1"/>
-      <c r="B9" s="1"/>
-      <c r="C9" s="1"/>
-      <c r="D9" s="1" t="s">
+      <c r="D9" t="s">
         <v>1</v>
       </c>
       <c r="E9">
@@ -2379,14 +2254,13 @@
       </c>
     </row>
     <row r="10" spans="1:6">
-      <c r="A10" s="1"/>
-      <c r="B10" s="1" t="s">
+      <c r="B10" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="C10" t="s">
         <v>31</v>
       </c>
-      <c r="D10" s="1" t="s">
+      <c r="D10" t="s">
         <v>0</v>
       </c>
       <c r="F10">
@@ -2394,10 +2268,7 @@
       </c>
     </row>
     <row r="11" spans="1:6">
-      <c r="A11" s="1"/>
-      <c r="B11" s="1"/>
-      <c r="C11" s="1"/>
-      <c r="D11" s="1" t="s">
+      <c r="D11" t="s">
         <v>1</v>
       </c>
       <c r="E11">
@@ -2405,14 +2276,13 @@
       </c>
     </row>
     <row r="12" spans="1:6">
-      <c r="A12" s="1"/>
-      <c r="B12" s="1" t="s">
+      <c r="B12" t="s">
         <v>15</v>
       </c>
-      <c r="C12" s="1" t="s">
+      <c r="C12" t="s">
         <v>31</v>
       </c>
-      <c r="D12" s="1" t="s">
+      <c r="D12" t="s">
         <v>0</v>
       </c>
       <c r="F12">
@@ -2420,10 +2290,7 @@
       </c>
     </row>
     <row r="13" spans="1:6">
-      <c r="A13" s="1"/>
-      <c r="B13" s="1"/>
-      <c r="C13" s="1"/>
-      <c r="D13" s="1" t="s">
+      <c r="D13" t="s">
         <v>1</v>
       </c>
       <c r="E13">
@@ -2431,14 +2298,13 @@
       </c>
     </row>
     <row r="14" spans="1:6">
-      <c r="A14" s="1"/>
-      <c r="B14" s="1" t="s">
+      <c r="B14" t="s">
         <v>16</v>
       </c>
-      <c r="C14" s="1" t="s">
+      <c r="C14" t="s">
         <v>25</v>
       </c>
-      <c r="D14" s="1" t="s">
+      <c r="D14" t="s">
         <v>0</v>
       </c>
       <c r="F14">
@@ -2446,10 +2312,7 @@
       </c>
     </row>
     <row r="15" spans="1:6">
-      <c r="A15" s="1"/>
-      <c r="B15" s="1"/>
-      <c r="C15" s="1"/>
-      <c r="D15" s="1" t="s">
+      <c r="D15" t="s">
         <v>1</v>
       </c>
       <c r="E15">
@@ -2457,155 +2320,131 @@
       </c>
     </row>
     <row r="16" spans="1:6">
-      <c r="A16" s="1"/>
-      <c r="B16" s="1" t="s">
+      <c r="B16" t="s">
         <v>17</v>
       </c>
-      <c r="C16" s="1" t="s">
+      <c r="C16" t="s">
         <v>25</v>
       </c>
-      <c r="D16" s="1" t="s">
+      <c r="D16" t="s">
         <v>0</v>
       </c>
       <c r="F16">
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:6">
-      <c r="A17" s="1"/>
-      <c r="B17" s="1"/>
-      <c r="C17" s="1"/>
-      <c r="D17" s="1" t="s">
+    <row r="17" spans="2:6">
+      <c r="D17" t="s">
         <v>1</v>
       </c>
       <c r="E17">
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:6">
-      <c r="A18" s="1"/>
-      <c r="B18" s="1" t="s">
+    <row r="18" spans="2:6">
+      <c r="B18" t="s">
         <v>19</v>
       </c>
-      <c r="C18" s="1" t="s">
+      <c r="C18" t="s">
         <v>32</v>
       </c>
-      <c r="D18" s="1" t="s">
+      <c r="D18" t="s">
         <v>0</v>
       </c>
       <c r="F18">
         <v>52560000</v>
       </c>
     </row>
-    <row r="19" spans="1:6">
-      <c r="A19" s="1"/>
-      <c r="B19" s="1"/>
-      <c r="C19" s="1"/>
-      <c r="D19" s="1" t="s">
+    <row r="19" spans="2:6">
+      <c r="D19" t="s">
         <v>1</v>
       </c>
       <c r="E19">
-        <v>4.52688691920903E-09</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6">
-      <c r="A20" s="1"/>
-      <c r="B20" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="2:6">
+      <c r="B20" t="s">
         <v>20</v>
       </c>
-      <c r="C20" s="1" t="s">
+      <c r="C20" t="s">
         <v>33</v>
       </c>
-      <c r="D20" s="1" t="s">
+      <c r="D20" t="s">
         <v>0</v>
       </c>
       <c r="F20">
         <v>52560000</v>
       </c>
     </row>
-    <row r="21" spans="1:6">
-      <c r="A21" s="1"/>
-      <c r="B21" s="1"/>
-      <c r="C21" s="1"/>
-      <c r="D21" s="1" t="s">
+    <row r="21" spans="2:6">
+      <c r="D21" t="s">
         <v>1</v>
       </c>
       <c r="E21">
-        <v>4.52688691920903E-09</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6">
-      <c r="A22" s="1"/>
-      <c r="B22" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="2:6">
+      <c r="B22" t="s">
         <v>21</v>
       </c>
-      <c r="C22" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D22" s="1" t="s">
+      <c r="C22" t="s">
+        <v>26</v>
+      </c>
+      <c r="D22" t="s">
         <v>0</v>
       </c>
       <c r="F22">
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:6">
-      <c r="A23" s="1"/>
-      <c r="B23" s="1"/>
-      <c r="C23" s="1"/>
-      <c r="D23" s="1" t="s">
+    <row r="23" spans="2:6">
+      <c r="D23" t="s">
         <v>1</v>
       </c>
       <c r="E23">
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:6">
-      <c r="A24" s="1"/>
-      <c r="B24" s="1" t="s">
+    <row r="24" spans="2:6">
+      <c r="B24" t="s">
         <v>23</v>
       </c>
-      <c r="C24" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D24" s="1" t="s">
+      <c r="C24" t="s">
+        <v>26</v>
+      </c>
+      <c r="D24" t="s">
         <v>0</v>
       </c>
       <c r="F24">
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:6">
-      <c r="A25" s="1"/>
-      <c r="B25" s="1"/>
-      <c r="C25" s="1"/>
-      <c r="D25" s="1" t="s">
+    <row r="25" spans="2:6">
+      <c r="D25" t="s">
         <v>1</v>
       </c>
       <c r="E25">
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:6">
-      <c r="A26" s="1"/>
-      <c r="B26" s="1" t="s">
+    <row r="26" spans="2:6">
+      <c r="B26" t="s">
         <v>24</v>
       </c>
-      <c r="C26" s="1" t="s">
+      <c r="C26" t="s">
         <v>25</v>
       </c>
-      <c r="D26" s="1" t="s">
+      <c r="D26" t="s">
         <v>0</v>
       </c>
       <c r="F26">
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:6">
-      <c r="A27" s="1"/>
-      <c r="B27" s="1"/>
-      <c r="C27" s="1"/>
-      <c r="D27" s="1" t="s">
+    <row r="27" spans="2:6">
+      <c r="D27" t="s">
         <v>1</v>
       </c>
       <c r="E27">

</xml_diff>

<commit_message>
Adapt to TSAM v4.0 (#827)
</commit_message>
<xml_diff>
--- a/test/data/expected_result_minisystem_segmentation.xlsx
+++ b/test/data/expected_result_minisystem_segmentation.xlsx
@@ -183,13 +183,13 @@
     <t>stateOfChargeOperationVariablesOptimum</t>
   </si>
   <si>
-    <t>LocationIn</t>
+    <t>locationIn</t>
   </si>
   <si>
     <t>Pipelines</t>
   </si>
   <si>
-    <t>LocationOut</t>
+    <t>locationOut</t>
   </si>
   <si>
     <t>periodsOrder</t>
@@ -205,16 +205,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -230,7 +222,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -238,30 +230,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -560,198 +534,182 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="E1" s="1" t="s">
+      <c r="D1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E1" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="1" t="s">
+      <c r="A2" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" t="s">
         <v>25</v>
       </c>
       <c r="D2">
-        <v>1520485.714285719</v>
+        <v>1708200.000000002</v>
       </c>
       <c r="E2">
         <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1" t="s">
+      <c r="B3" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" t="s">
         <v>26</v>
       </c>
       <c r="D3">
-        <v>1520485.714285718</v>
+        <v>1708200</v>
       </c>
       <c r="E3">
         <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="1"/>
-      <c r="B4" s="1" t="s">
+      <c r="B4" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="1"/>
-      <c r="B5" s="1" t="s">
+      <c r="B5" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="1"/>
-      <c r="B6" s="1" t="s">
+      <c r="B6" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="1"/>
-      <c r="B7" s="1" t="s">
+      <c r="B7" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="C7" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="1"/>
-      <c r="B8" s="1" t="s">
+      <c r="B8" t="s">
         <v>13</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="C8" t="s">
         <v>26</v>
       </c>
       <c r="D8">
-        <v>1895914.285714289</v>
+        <v>1895914.285714286</v>
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="1"/>
-      <c r="B9" s="1" t="s">
+      <c r="B9" t="s">
         <v>14</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="C9" t="s">
         <v>26</v>
       </c>
       <c r="D9">
-        <v>375428.571428571</v>
+        <v>187714.2857142857</v>
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="1"/>
-      <c r="B10" s="1" t="s">
+      <c r="B10" t="s">
         <v>15</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="C10" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="1"/>
-      <c r="B11" s="1" t="s">
+      <c r="B11" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="C11" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="1"/>
-      <c r="B12" s="1" t="s">
+      <c r="B12" t="s">
         <v>17</v>
       </c>
-      <c r="C12" s="1" t="s">
+      <c r="C12" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="1"/>
-      <c r="B13" s="1" t="s">
+      <c r="B13" t="s">
         <v>18</v>
       </c>
-      <c r="C13" s="1" t="s">
+      <c r="C13" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="1"/>
-      <c r="B14" s="1" t="s">
+      <c r="B14" t="s">
         <v>19</v>
       </c>
-      <c r="C14" s="1" t="s">
+      <c r="C14" t="s">
         <v>29</v>
       </c>
       <c r="D14">
-        <v>75085714.2857143</v>
+        <v>75085714.28571428</v>
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="1"/>
-      <c r="B15" s="1" t="s">
+      <c r="B15" t="s">
         <v>20</v>
       </c>
-      <c r="C15" s="1" t="s">
+      <c r="C15" t="s">
         <v>30</v>
       </c>
       <c r="D15">
-        <v>75085714.2857143</v>
+        <v>75085714.28571428</v>
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="1"/>
-      <c r="B16" s="1" t="s">
+      <c r="B16" t="s">
         <v>21</v>
       </c>
-      <c r="C16" s="1" t="s">
+      <c r="C16" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="1"/>
-      <c r="B17" s="1" t="s">
+      <c r="B17" t="s">
         <v>22</v>
       </c>
-      <c r="C17" s="1" t="s">
+      <c r="C17" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="1"/>
-      <c r="B18" s="1" t="s">
+      <c r="B18" t="s">
         <v>23</v>
       </c>
-      <c r="C18" s="1" t="s">
+      <c r="C18" t="s">
         <v>26</v>
       </c>
       <c r="D18">
@@ -759,22 +717,21 @@
       </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="1"/>
-      <c r="B19" s="1" t="s">
+      <c r="B19" t="s">
         <v>24</v>
       </c>
-      <c r="C19" s="1" t="s">
+      <c r="C19" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="1" t="s">
+      <c r="A20" t="s">
         <v>6</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="B20" t="s">
         <v>7</v>
       </c>
-      <c r="C20" s="1" t="s">
+      <c r="C20" t="s">
         <v>25</v>
       </c>
       <c r="D20">
@@ -785,11 +742,10 @@
       </c>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="1"/>
-      <c r="B21" s="1" t="s">
+      <c r="B21" t="s">
         <v>8</v>
       </c>
-      <c r="C21" s="1" t="s">
+      <c r="C21" t="s">
         <v>26</v>
       </c>
       <c r="D21">
@@ -800,47 +756,42 @@
       </c>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="1"/>
-      <c r="B22" s="1" t="s">
+      <c r="B22" t="s">
         <v>9</v>
       </c>
-      <c r="C22" s="1" t="s">
+      <c r="C22" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="23" spans="1:5">
-      <c r="A23" s="1"/>
-      <c r="B23" s="1" t="s">
+      <c r="B23" t="s">
         <v>10</v>
       </c>
-      <c r="C23" s="1" t="s">
+      <c r="C23" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="24" spans="1:5">
-      <c r="A24" s="1"/>
-      <c r="B24" s="1" t="s">
+      <c r="B24" t="s">
         <v>11</v>
       </c>
-      <c r="C24" s="1" t="s">
+      <c r="C24" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="25" spans="1:5">
-      <c r="A25" s="1"/>
-      <c r="B25" s="1" t="s">
+      <c r="B25" t="s">
         <v>12</v>
       </c>
-      <c r="C25" s="1" t="s">
+      <c r="C25" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="1"/>
-      <c r="B26" s="1" t="s">
+      <c r="B26" t="s">
         <v>13</v>
       </c>
-      <c r="C26" s="1" t="s">
+      <c r="C26" t="s">
         <v>26</v>
       </c>
       <c r="E26">
@@ -848,11 +799,10 @@
       </c>
     </row>
     <row r="27" spans="1:5">
-      <c r="A27" s="1"/>
-      <c r="B27" s="1" t="s">
+      <c r="B27" t="s">
         <v>14</v>
       </c>
-      <c r="C27" s="1" t="s">
+      <c r="C27" t="s">
         <v>26</v>
       </c>
       <c r="E27">
@@ -860,101 +810,91 @@
       </c>
     </row>
     <row r="28" spans="1:5">
-      <c r="A28" s="1"/>
-      <c r="B28" s="1" t="s">
+      <c r="B28" t="s">
         <v>15</v>
       </c>
-      <c r="C28" s="1" t="s">
+      <c r="C28" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="29" spans="1:5">
-      <c r="A29" s="1"/>
-      <c r="B29" s="1" t="s">
+      <c r="B29" t="s">
         <v>16</v>
       </c>
-      <c r="C29" s="1" t="s">
+      <c r="C29" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="30" spans="1:5">
-      <c r="A30" s="1"/>
-      <c r="B30" s="1" t="s">
+      <c r="B30" t="s">
         <v>17</v>
       </c>
-      <c r="C30" s="1" t="s">
+      <c r="C30" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="31" spans="1:5">
-      <c r="A31" s="1"/>
-      <c r="B31" s="1" t="s">
+      <c r="B31" t="s">
         <v>18</v>
       </c>
-      <c r="C31" s="1" t="s">
+      <c r="C31" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="32" spans="1:5">
-      <c r="A32" s="1"/>
-      <c r="B32" s="1" t="s">
+      <c r="B32" t="s">
         <v>19</v>
       </c>
-      <c r="C32" s="1" t="s">
+      <c r="C32" t="s">
         <v>32</v>
       </c>
       <c r="E32">
         <v>52560000</v>
       </c>
     </row>
-    <row r="33" spans="1:5">
-      <c r="A33" s="1"/>
-      <c r="B33" s="1" t="s">
+    <row r="33" spans="2:5">
+      <c r="B33" t="s">
         <v>20</v>
       </c>
-      <c r="C33" s="1" t="s">
+      <c r="C33" t="s">
         <v>33</v>
       </c>
       <c r="E33">
         <v>52560000</v>
       </c>
     </row>
-    <row r="34" spans="1:5">
-      <c r="A34" s="1"/>
-      <c r="B34" s="1" t="s">
+    <row r="34" spans="2:5">
+      <c r="B34" t="s">
         <v>21</v>
       </c>
-      <c r="C34" s="1" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5">
-      <c r="A35" s="1"/>
-      <c r="B35" s="1" t="s">
+      <c r="C34" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="35" spans="2:5">
+      <c r="B35" t="s">
         <v>22</v>
       </c>
-      <c r="C35" s="1" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5">
-      <c r="A36" s="1"/>
-      <c r="B36" s="1" t="s">
+      <c r="C35" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="36" spans="2:5">
+      <c r="B36" t="s">
         <v>23</v>
       </c>
-      <c r="C36" s="1" t="s">
+      <c r="C36" t="s">
         <v>26</v>
       </c>
       <c r="E36">
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:5">
-      <c r="A37" s="1"/>
-      <c r="B37" s="1" t="s">
+    <row r="37" spans="2:5">
+      <c r="B37" t="s">
         <v>24</v>
       </c>
-      <c r="C37" s="1" t="s">
+      <c r="C37" t="s">
         <v>25</v>
       </c>
     </row>
@@ -973,42 +913,42 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>34</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>52</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>54</v>
       </c>
-      <c r="E1" s="1">
-        <v>0</v>
-      </c>
-      <c r="F1" s="1">
-        <v>1</v>
-      </c>
-      <c r="G1" s="1">
+      <c r="E1">
+        <v>0</v>
+      </c>
+      <c r="F1">
+        <v>1</v>
+      </c>
+      <c r="G1">
         <v>2</v>
       </c>
-      <c r="H1" s="1">
+      <c r="H1">
         <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:8">
-      <c r="A2" s="1" t="s">
+      <c r="A2" t="s">
         <v>36</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" t="s">
         <v>53</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D2" s="1" t="s">
+      <c r="C2" t="s">
+        <v>0</v>
+      </c>
+      <c r="D2" t="s">
         <v>1</v>
       </c>
       <c r="E2">
@@ -1025,25 +965,23 @@
       </c>
     </row>
     <row r="3" spans="1:8">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D3" s="1" t="s">
+      <c r="C3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D3" t="s">
         <v>0</v>
       </c>
       <c r="E3">
-        <v>1.50896230640301E-09</v>
+        <v>0</v>
       </c>
       <c r="F3">
         <v>0</v>
       </c>
       <c r="G3">
-        <v>1.50896230640301E-09</v>
+        <v>0</v>
       </c>
       <c r="H3">
-        <v>1.50896230640301E-09</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1061,30 +999,30 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>35</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="E1" s="1" t="s">
+      <c r="D1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E1" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="1" t="s">
+      <c r="A2" t="s">
         <v>39</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" t="s">
         <v>53</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" t="s">
         <v>0</v>
       </c>
       <c r="E2">
@@ -1092,9 +1030,7 @@
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1" t="s">
+      <c r="C3" t="s">
         <v>1</v>
       </c>
       <c r="D3">
@@ -1102,13 +1038,13 @@
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="1" t="s">
+      <c r="A4" t="s">
         <v>40</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" t="s">
         <v>53</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" t="s">
         <v>0</v>
       </c>
       <c r="E4">
@@ -1116,9 +1052,7 @@
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="1"/>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1" t="s">
+      <c r="C5" t="s">
         <v>1</v>
       </c>
       <c r="D5">
@@ -1126,13 +1060,13 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="1" t="s">
+      <c r="A6" t="s">
         <v>41</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" t="s">
         <v>53</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" t="s">
         <v>0</v>
       </c>
       <c r="E6">
@@ -1140,9 +1074,7 @@
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="1"/>
-      <c r="B7" s="1"/>
-      <c r="C7" s="1" t="s">
+      <c r="C7" t="s">
         <v>1</v>
       </c>
       <c r="D7">
@@ -1168,15 +1100,15 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="B1" s="1">
-        <v>0</v>
-      </c>
-      <c r="C1" s="1">
+      <c r="B1">
+        <v>0</v>
+      </c>
+      <c r="C1">
         <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:3">
-      <c r="A2" s="1" t="s">
+      <c r="A2" t="s">
         <v>55</v>
       </c>
       <c r="B2">
@@ -1187,18 +1119,18 @@
       </c>
     </row>
     <row r="4" spans="1:3">
-      <c r="A4" s="1" t="s">
+      <c r="A4" t="s">
         <v>57</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" t="s">
         <v>56</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="5" spans="1:3">
-      <c r="A5" s="1">
+      <c r="A5">
         <v>0</v>
       </c>
       <c r="B5">
@@ -1209,7 +1141,7 @@
       </c>
     </row>
     <row r="6" spans="1:3">
-      <c r="A6" s="1">
+      <c r="A6">
         <v>1</v>
       </c>
       <c r="B6">
@@ -1230,57 +1162,56 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>34</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>35</v>
       </c>
-      <c r="D1" s="1">
-        <v>0</v>
-      </c>
-      <c r="E1" s="1">
-        <v>1</v>
-      </c>
-      <c r="F1" s="1">
+      <c r="D1">
+        <v>0</v>
+      </c>
+      <c r="E1">
+        <v>1</v>
+      </c>
+      <c r="F1">
         <v>2</v>
       </c>
-      <c r="G1" s="1">
+      <c r="G1">
         <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:7">
-      <c r="A2" s="1" t="s">
+      <c r="A2" t="s">
         <v>36</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" t="s">
         <v>0</v>
       </c>
       <c r="D2">
-        <v>18771428.5714286</v>
+        <v>37542857.14285714</v>
       </c>
       <c r="E2">
-        <v>37542857.1428571</v>
+        <v>18771428.57142857</v>
       </c>
       <c r="F2">
-        <v>0</v>
+        <v>18771428.57142857</v>
       </c>
       <c r="G2">
-        <v>18771428.5714286</v>
+        <v>-0</v>
       </c>
     </row>
     <row r="3" spans="1:7">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1" t="s">
+      <c r="B3" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" t="s">
         <v>1</v>
       </c>
       <c r="D3">
@@ -1310,114 +1241,108 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="E1" s="1" t="s">
+      <c r="D1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E1" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="1" t="s">
+      <c r="A2" t="s">
         <v>37</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" t="s">
         <v>25</v>
       </c>
       <c r="D2">
-        <v>1491681.331689215</v>
+        <v>1491681.331689218</v>
       </c>
       <c r="E2">
         <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1" t="s">
+      <c r="B3" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" t="s">
         <v>26</v>
       </c>
       <c r="D3">
-        <v>1491681.331689214</v>
+        <v>1491681.331689217</v>
       </c>
       <c r="E3">
         <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="1"/>
-      <c r="B4" s="1" t="s">
+      <c r="B4" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" t="s">
         <v>27</v>
       </c>
       <c r="D4">
-        <v>17142.8571428571</v>
+        <v>17142.85714285714</v>
       </c>
       <c r="E4">
         <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="1"/>
-      <c r="B5" s="1" t="s">
+      <c r="B5" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" t="s">
         <v>26</v>
       </c>
       <c r="D5">
-        <v>1277395.6174035</v>
+        <v>1277395.617403503</v>
       </c>
       <c r="E5">
         <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="1"/>
-      <c r="B6" s="1" t="s">
+      <c r="B6" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="1"/>
-      <c r="B7" s="1" t="s">
+      <c r="B7" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="C7" t="s">
         <v>27</v>
       </c>
       <c r="D7">
-        <v>17142.8571428571</v>
+        <v>17142.85714285714</v>
       </c>
       <c r="E7">
         <v>-0</v>
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="1"/>
-      <c r="B8" s="1" t="s">
+      <c r="B8" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="C8" t="s">
         <v>27</v>
       </c>
       <c r="D8">
@@ -1428,26 +1353,24 @@
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="1"/>
-      <c r="B9" s="1" t="s">
+      <c r="B9" t="s">
         <v>16</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="C9" t="s">
         <v>25</v>
       </c>
       <c r="D9">
-        <v>8571428.57142855</v>
+        <v>8571428.571428571</v>
       </c>
       <c r="E9">
         <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="1"/>
-      <c r="B10" s="1" t="s">
+      <c r="B10" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="C10" t="s">
         <v>25</v>
       </c>
       <c r="D10">
@@ -1458,74 +1381,68 @@
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="1"/>
-      <c r="B11" s="1" t="s">
+      <c r="B11" t="s">
         <v>18</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="C11" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="1"/>
-      <c r="B12" s="1" t="s">
+      <c r="B12" t="s">
         <v>19</v>
       </c>
-      <c r="C12" s="1" t="s">
+      <c r="C12" t="s">
         <v>29</v>
       </c>
       <c r="D12">
-        <v>75085714.2857143</v>
+        <v>75085714.28571428</v>
       </c>
       <c r="E12">
         <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="1"/>
-      <c r="B13" s="1" t="s">
+      <c r="B13" t="s">
         <v>20</v>
       </c>
-      <c r="C13" s="1" t="s">
+      <c r="C13" t="s">
         <v>30</v>
       </c>
       <c r="D13">
-        <v>75085714.2857143</v>
+        <v>75085714.28571428</v>
       </c>
       <c r="E13">
         <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="1"/>
-      <c r="B14" s="1" t="s">
+      <c r="B14" t="s">
         <v>21</v>
       </c>
-      <c r="C14" s="1" t="s">
+      <c r="C14" t="s">
         <v>26</v>
       </c>
       <c r="D14">
-        <v>214285.7142857138</v>
+        <v>214285.7142857143</v>
       </c>
       <c r="E14">
         <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="1"/>
-      <c r="B15" s="1" t="s">
+      <c r="B15" t="s">
         <v>22</v>
       </c>
-      <c r="C15" s="1" t="s">
+      <c r="C15" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="1"/>
-      <c r="B16" s="1" t="s">
+      <c r="B16" t="s">
         <v>23</v>
       </c>
-      <c r="C16" s="1" t="s">
+      <c r="C16" t="s">
         <v>26</v>
       </c>
       <c r="D16">
@@ -1535,12 +1452,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:5">
-      <c r="A17" s="1"/>
-      <c r="B17" s="1" t="s">
+    <row r="17" spans="2:5">
+      <c r="B17" t="s">
         <v>24</v>
       </c>
-      <c r="C17" s="1" t="s">
+      <c r="C17" t="s">
         <v>25</v>
       </c>
       <c r="D17">
@@ -1564,68 +1480,66 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>34</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>35</v>
       </c>
-      <c r="D1" s="1">
-        <v>0</v>
-      </c>
-      <c r="E1" s="1">
-        <v>1</v>
-      </c>
-      <c r="F1" s="1">
+      <c r="D1">
+        <v>0</v>
+      </c>
+      <c r="E1">
+        <v>1</v>
+      </c>
+      <c r="F1">
         <v>2</v>
       </c>
-      <c r="G1" s="1">
+      <c r="G1">
         <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:7">
-      <c r="A2" s="1" t="s">
+      <c r="A2" t="s">
         <v>36</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" t="s">
         <v>37</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" t="s">
         <v>0</v>
       </c>
       <c r="D2">
-        <v>18771428.5714286</v>
+        <v>37542857.14285714</v>
       </c>
       <c r="E2">
-        <v>37542857.1428571</v>
+        <v>18771428.57142857</v>
       </c>
       <c r="F2">
-        <v>0</v>
+        <v>18771428.57142857</v>
       </c>
       <c r="G2">
-        <v>18771428.5714286</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:7">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1" t="s">
+      <c r="C3" t="s">
         <v>1</v>
       </c>
       <c r="D3">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="F3">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="G3">
-        <v>0</v>
+        <v>-0</v>
       </c>
     </row>
   </sheetData>
@@ -1643,52 +1557,52 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1" s="1" t="s">
+      <c r="C1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:4">
-      <c r="A2" s="1" t="s">
+      <c r="A2" t="s">
         <v>39</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" t="s">
         <v>37</v>
       </c>
       <c r="C2">
-        <v>17142.8571428571</v>
+        <v>17142.85714285714</v>
       </c>
       <c r="D2">
         <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:4">
-      <c r="A3" s="1" t="s">
+      <c r="A3" t="s">
         <v>40</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" t="s">
         <v>37</v>
       </c>
       <c r="C3">
-        <v>17142.8571428571</v>
+        <v>17142.85714285714</v>
       </c>
       <c r="D3">
         <v>-0</v>
       </c>
     </row>
     <row r="4" spans="1:4">
-      <c r="A4" s="1" t="s">
+      <c r="A4" t="s">
         <v>41</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" t="s">
         <v>37</v>
       </c>
       <c r="C4">
@@ -1709,114 +1623,108 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="E1" s="1" t="s">
+      <c r="D1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E1" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="1" t="s">
+      <c r="A2" t="s">
         <v>42</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" t="s">
         <v>25</v>
       </c>
       <c r="D2">
-        <v>871039.1602304186</v>
+        <v>871039.1602304169</v>
       </c>
       <c r="E2">
-        <v>1.000277975790437E-10</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1" t="s">
+      <c r="B3" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" t="s">
         <v>26</v>
       </c>
       <c r="D3">
-        <v>871039.1602304177</v>
+        <v>871039.1602304161</v>
       </c>
       <c r="E3">
-        <v>1.000277975790436E-10</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="1"/>
-      <c r="B4" s="1" t="s">
+      <c r="B4" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" t="s">
         <v>32</v>
       </c>
       <c r="D4">
-        <v>19611940.2985075</v>
+        <v>19611940.29850746</v>
       </c>
       <c r="E4">
-        <v>2.25218254687017E-09</v>
+        <v>-0</v>
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="1"/>
-      <c r="B5" s="1" t="s">
+      <c r="B5" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" t="s">
         <v>26</v>
       </c>
       <c r="D5">
-        <v>871039.1602304177</v>
+        <v>871039.1602304161</v>
       </c>
       <c r="E5">
-        <v>1.000277975790436E-10</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="1"/>
-      <c r="B6" s="1" t="s">
+      <c r="B6" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="1"/>
-      <c r="B7" s="1" t="s">
+      <c r="B7" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="C7" t="s">
         <v>32</v>
       </c>
       <c r="D7">
-        <v>19611940.2985075</v>
+        <v>19611940.29850746</v>
       </c>
       <c r="E7">
-        <v>2.25218254687017E-09</v>
+        <v>-0</v>
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="1"/>
-      <c r="B8" s="1" t="s">
+      <c r="B8" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="C8" t="s">
         <v>32</v>
       </c>
       <c r="D8">
@@ -1827,26 +1735,24 @@
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="1"/>
-      <c r="B9" s="1" t="s">
+      <c r="B9" t="s">
         <v>16</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="C9" t="s">
         <v>25</v>
       </c>
       <c r="D9">
-        <v>9805970.14925375</v>
+        <v>9805970.149253732</v>
       </c>
       <c r="E9">
-        <v>1.126091273435085E-09</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="1"/>
-      <c r="B10" s="1" t="s">
+      <c r="B10" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="C10" t="s">
         <v>25</v>
       </c>
       <c r="D10">
@@ -1857,80 +1763,74 @@
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="1"/>
-      <c r="B11" s="1" t="s">
+      <c r="B11" t="s">
         <v>18</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="C11" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="1"/>
-      <c r="B12" s="1" t="s">
+      <c r="B12" t="s">
         <v>43</v>
       </c>
-      <c r="C12" s="1" t="s">
+      <c r="C12" t="s">
         <v>32</v>
       </c>
       <c r="D12">
         <v>13140000</v>
       </c>
       <c r="E12">
-        <v>1.50896230640301E-09</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="1"/>
-      <c r="B13" s="1" t="s">
+      <c r="B13" t="s">
         <v>44</v>
       </c>
-      <c r="C13" s="1" t="s">
+      <c r="C13" t="s">
         <v>33</v>
       </c>
       <c r="D13">
         <v>13140000</v>
       </c>
       <c r="E13">
-        <v>1.50896230640301E-09</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="1"/>
-      <c r="B14" s="1" t="s">
+      <c r="B14" t="s">
         <v>45</v>
       </c>
-      <c r="C14" s="1" t="s">
+      <c r="C14" t="s">
         <v>32</v>
       </c>
       <c r="D14">
         <v>13140000</v>
       </c>
       <c r="E14">
-        <v>1.50896230640301E-09</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="1"/>
-      <c r="B15" s="1" t="s">
+      <c r="B15" t="s">
         <v>46</v>
       </c>
-      <c r="C15" s="1" t="s">
+      <c r="C15" t="s">
         <v>33</v>
       </c>
       <c r="D15">
         <v>13140000</v>
       </c>
       <c r="E15">
-        <v>1.50896230640301E-09</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="1"/>
-      <c r="B16" s="1" t="s">
+      <c r="B16" t="s">
         <v>21</v>
       </c>
-      <c r="C16" s="1" t="s">
+      <c r="C16" t="s">
         <v>26</v>
       </c>
       <c r="D16">
@@ -1940,12 +1840,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:5">
-      <c r="A17" s="1"/>
-      <c r="B17" s="1" t="s">
+    <row r="17" spans="2:5">
+      <c r="B17" t="s">
         <v>47</v>
       </c>
-      <c r="C17" s="1" t="s">
+      <c r="C17" t="s">
         <v>26</v>
       </c>
       <c r="D17">
@@ -1955,12 +1854,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:5">
-      <c r="A18" s="1"/>
-      <c r="B18" s="1" t="s">
+    <row r="18" spans="2:5">
+      <c r="B18" t="s">
         <v>48</v>
       </c>
-      <c r="C18" s="1" t="s">
+      <c r="C18" t="s">
         <v>26</v>
       </c>
       <c r="D18">
@@ -1970,21 +1868,19 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:5">
-      <c r="A19" s="1"/>
-      <c r="B19" s="1" t="s">
+    <row r="19" spans="2:5">
+      <c r="B19" t="s">
         <v>22</v>
       </c>
-      <c r="C19" s="1" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5">
-      <c r="A20" s="1"/>
-      <c r="B20" s="1" t="s">
+      <c r="C19" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="20" spans="2:5">
+      <c r="B20" t="s">
         <v>24</v>
       </c>
-      <c r="C20" s="1" t="s">
+      <c r="C20" t="s">
         <v>25</v>
       </c>
       <c r="D20">
@@ -2008,152 +1904,146 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>34</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>35</v>
       </c>
-      <c r="D1" s="1">
-        <v>0</v>
-      </c>
-      <c r="E1" s="1">
-        <v>1</v>
-      </c>
-      <c r="F1" s="1">
+      <c r="D1">
+        <v>0</v>
+      </c>
+      <c r="E1">
+        <v>1</v>
+      </c>
+      <c r="F1">
         <v>2</v>
       </c>
-      <c r="G1" s="1">
+      <c r="G1">
         <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:7">
-      <c r="A2" s="1" t="s">
+      <c r="A2" t="s">
         <v>49</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" t="s">
         <v>42</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" t="s">
         <v>0</v>
       </c>
       <c r="D2">
-        <v>0</v>
+        <v>13140000</v>
       </c>
       <c r="E2">
+        <v>0</v>
+      </c>
+      <c r="F2">
+        <v>-0</v>
+      </c>
+      <c r="G2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
+      <c r="C3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>-0</v>
+      </c>
+      <c r="E3">
+        <v>0</v>
+      </c>
+      <c r="F3">
+        <v>-0</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B4" t="s">
+        <v>42</v>
+      </c>
+      <c r="C4" t="s">
+        <v>0</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>-0</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4">
         <v>13140000</v>
       </c>
-      <c r="F2">
-        <v>0</v>
-      </c>
-      <c r="G2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D3">
-        <v>0</v>
-      </c>
-      <c r="E3">
-        <v>1.50896230640301E-09</v>
-      </c>
-      <c r="F3">
-        <v>0</v>
-      </c>
-      <c r="G3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7">
-      <c r="A4" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="B4" s="1" t="s">
+    </row>
+    <row r="5" spans="1:7">
+      <c r="C5" t="s">
+        <v>1</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5">
+        <v>-0</v>
+      </c>
+      <c r="F5">
+        <v>0</v>
+      </c>
+      <c r="G5">
+        <v>-0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B6" t="s">
         <v>42</v>
       </c>
-      <c r="C4" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D4">
-        <v>0</v>
-      </c>
-      <c r="E4">
-        <v>0</v>
-      </c>
-      <c r="F4">
-        <v>13140000</v>
-      </c>
-      <c r="G4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7">
-      <c r="A5" s="1"/>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D5">
-        <v>0</v>
-      </c>
-      <c r="E5">
-        <v>0</v>
-      </c>
-      <c r="F5">
-        <v>1.50896230640301E-09</v>
-      </c>
-      <c r="G5">
-        <v>5.13302352179869E-25</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7">
-      <c r="A6" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" t="s">
         <v>0</v>
       </c>
       <c r="D6">
-        <v>6471940.29850747</v>
+        <v>6471940.298507463</v>
       </c>
       <c r="E6">
-        <v>6471940.29850747</v>
+        <v>19611940.29850746</v>
       </c>
       <c r="F6">
-        <v>19611940.2985075</v>
+        <v>19611940.29850746</v>
       </c>
       <c r="G6">
-        <v>6471940.2985075</v>
+        <v>19611940.29850746</v>
       </c>
     </row>
     <row r="7" spans="1:7">
-      <c r="A7" s="1"/>
-      <c r="B7" s="1"/>
-      <c r="C7" s="1" t="s">
+      <c r="C7" t="s">
         <v>1</v>
       </c>
       <c r="D7">
-        <v>7.43220240467156E-10</v>
+        <v>0</v>
       </c>
       <c r="E7">
-        <v>7.43220240467156E-10</v>
+        <v>-0</v>
       </c>
       <c r="F7">
-        <v>2.25218254687017E-09</v>
+        <v>0</v>
       </c>
       <c r="G7">
-        <v>7.432202404671603E-10</v>
+        <v>-0</v>
       </c>
     </row>
   </sheetData>
@@ -2175,59 +2065,59 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1" s="1" t="s">
+      <c r="C1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:4">
-      <c r="A2" s="1" t="s">
+      <c r="A2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C2">
+        <v>19611940.29850746</v>
+      </c>
+      <c r="D2">
+        <v>-0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" t="s">
         <v>40</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B3" t="s">
         <v>42</v>
       </c>
-      <c r="C2">
-        <v>19611940.2985075</v>
-      </c>
-      <c r="D2">
-        <v>2.25218254687017E-09</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4">
-      <c r="A3" s="1" t="s">
+      <c r="C3">
+        <v>19611940.29850746</v>
+      </c>
+      <c r="D3">
+        <v>-0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" t="s">
         <v>41</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B4" t="s">
         <v>42</v>
       </c>
-      <c r="C3">
-        <v>0</v>
-      </c>
-      <c r="D3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4">
-      <c r="A4" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>42</v>
-      </c>
       <c r="C4">
-        <v>19611940.2985075</v>
+        <v>0</v>
       </c>
       <c r="D4">
-        <v>2.25218254687017E-09</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -2241,36 +2131,36 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>52</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="F1" s="1" t="s">
+      <c r="E1" t="s">
+        <v>0</v>
+      </c>
+      <c r="F1" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:6">
-      <c r="A2" s="1" t="s">
+      <c r="A2" t="s">
         <v>53</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" t="s">
         <v>25</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" t="s">
         <v>0</v>
       </c>
       <c r="E2">
@@ -2281,10 +2171,7 @@
       </c>
     </row>
     <row r="3" spans="1:6">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1" t="s">
+      <c r="D3" t="s">
         <v>1</v>
       </c>
       <c r="E3">
@@ -2295,14 +2182,13 @@
       </c>
     </row>
     <row r="4" spans="1:6">
-      <c r="A4" s="1"/>
-      <c r="B4" s="1" t="s">
+      <c r="B4" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D4" s="1" t="s">
+      <c r="C4" t="s">
+        <v>26</v>
+      </c>
+      <c r="D4" t="s">
         <v>0</v>
       </c>
       <c r="E4">
@@ -2313,10 +2199,7 @@
       </c>
     </row>
     <row r="5" spans="1:6">
-      <c r="A5" s="1"/>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1" t="s">
+      <c r="D5" t="s">
         <v>1</v>
       </c>
       <c r="E5">
@@ -2327,14 +2210,13 @@
       </c>
     </row>
     <row r="6" spans="1:6">
-      <c r="A6" s="1"/>
-      <c r="B6" s="1" t="s">
+      <c r="B6" t="s">
         <v>9</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" t="s">
         <v>31</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="D6" t="s">
         <v>0</v>
       </c>
       <c r="F6">
@@ -2342,10 +2224,7 @@
       </c>
     </row>
     <row r="7" spans="1:6">
-      <c r="A7" s="1"/>
-      <c r="B7" s="1"/>
-      <c r="C7" s="1"/>
-      <c r="D7" s="1" t="s">
+      <c r="D7" t="s">
         <v>1</v>
       </c>
       <c r="E7">
@@ -2353,14 +2232,13 @@
       </c>
     </row>
     <row r="8" spans="1:6">
-      <c r="A8" s="1"/>
-      <c r="B8" s="1" t="s">
+      <c r="B8" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D8" s="1" t="s">
+      <c r="C8" t="s">
+        <v>26</v>
+      </c>
+      <c r="D8" t="s">
         <v>0</v>
       </c>
       <c r="F8">
@@ -2368,10 +2246,7 @@
       </c>
     </row>
     <row r="9" spans="1:6">
-      <c r="A9" s="1"/>
-      <c r="B9" s="1"/>
-      <c r="C9" s="1"/>
-      <c r="D9" s="1" t="s">
+      <c r="D9" t="s">
         <v>1</v>
       </c>
       <c r="E9">
@@ -2379,14 +2254,13 @@
       </c>
     </row>
     <row r="10" spans="1:6">
-      <c r="A10" s="1"/>
-      <c r="B10" s="1" t="s">
+      <c r="B10" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="C10" t="s">
         <v>31</v>
       </c>
-      <c r="D10" s="1" t="s">
+      <c r="D10" t="s">
         <v>0</v>
       </c>
       <c r="F10">
@@ -2394,10 +2268,7 @@
       </c>
     </row>
     <row r="11" spans="1:6">
-      <c r="A11" s="1"/>
-      <c r="B11" s="1"/>
-      <c r="C11" s="1"/>
-      <c r="D11" s="1" t="s">
+      <c r="D11" t="s">
         <v>1</v>
       </c>
       <c r="E11">
@@ -2405,14 +2276,13 @@
       </c>
     </row>
     <row r="12" spans="1:6">
-      <c r="A12" s="1"/>
-      <c r="B12" s="1" t="s">
+      <c r="B12" t="s">
         <v>15</v>
       </c>
-      <c r="C12" s="1" t="s">
+      <c r="C12" t="s">
         <v>31</v>
       </c>
-      <c r="D12" s="1" t="s">
+      <c r="D12" t="s">
         <v>0</v>
       </c>
       <c r="F12">
@@ -2420,10 +2290,7 @@
       </c>
     </row>
     <row r="13" spans="1:6">
-      <c r="A13" s="1"/>
-      <c r="B13" s="1"/>
-      <c r="C13" s="1"/>
-      <c r="D13" s="1" t="s">
+      <c r="D13" t="s">
         <v>1</v>
       </c>
       <c r="E13">
@@ -2431,14 +2298,13 @@
       </c>
     </row>
     <row r="14" spans="1:6">
-      <c r="A14" s="1"/>
-      <c r="B14" s="1" t="s">
+      <c r="B14" t="s">
         <v>16</v>
       </c>
-      <c r="C14" s="1" t="s">
+      <c r="C14" t="s">
         <v>25</v>
       </c>
-      <c r="D14" s="1" t="s">
+      <c r="D14" t="s">
         <v>0</v>
       </c>
       <c r="F14">
@@ -2446,10 +2312,7 @@
       </c>
     </row>
     <row r="15" spans="1:6">
-      <c r="A15" s="1"/>
-      <c r="B15" s="1"/>
-      <c r="C15" s="1"/>
-      <c r="D15" s="1" t="s">
+      <c r="D15" t="s">
         <v>1</v>
       </c>
       <c r="E15">
@@ -2457,155 +2320,131 @@
       </c>
     </row>
     <row r="16" spans="1:6">
-      <c r="A16" s="1"/>
-      <c r="B16" s="1" t="s">
+      <c r="B16" t="s">
         <v>17</v>
       </c>
-      <c r="C16" s="1" t="s">
+      <c r="C16" t="s">
         <v>25</v>
       </c>
-      <c r="D16" s="1" t="s">
+      <c r="D16" t="s">
         <v>0</v>
       </c>
       <c r="F16">
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:6">
-      <c r="A17" s="1"/>
-      <c r="B17" s="1"/>
-      <c r="C17" s="1"/>
-      <c r="D17" s="1" t="s">
+    <row r="17" spans="2:6">
+      <c r="D17" t="s">
         <v>1</v>
       </c>
       <c r="E17">
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:6">
-      <c r="A18" s="1"/>
-      <c r="B18" s="1" t="s">
+    <row r="18" spans="2:6">
+      <c r="B18" t="s">
         <v>19</v>
       </c>
-      <c r="C18" s="1" t="s">
+      <c r="C18" t="s">
         <v>32</v>
       </c>
-      <c r="D18" s="1" t="s">
+      <c r="D18" t="s">
         <v>0</v>
       </c>
       <c r="F18">
         <v>52560000</v>
       </c>
     </row>
-    <row r="19" spans="1:6">
-      <c r="A19" s="1"/>
-      <c r="B19" s="1"/>
-      <c r="C19" s="1"/>
-      <c r="D19" s="1" t="s">
+    <row r="19" spans="2:6">
+      <c r="D19" t="s">
         <v>1</v>
       </c>
       <c r="E19">
-        <v>4.52688691920903E-09</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6">
-      <c r="A20" s="1"/>
-      <c r="B20" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="2:6">
+      <c r="B20" t="s">
         <v>20</v>
       </c>
-      <c r="C20" s="1" t="s">
+      <c r="C20" t="s">
         <v>33</v>
       </c>
-      <c r="D20" s="1" t="s">
+      <c r="D20" t="s">
         <v>0</v>
       </c>
       <c r="F20">
         <v>52560000</v>
       </c>
     </row>
-    <row r="21" spans="1:6">
-      <c r="A21" s="1"/>
-      <c r="B21" s="1"/>
-      <c r="C21" s="1"/>
-      <c r="D21" s="1" t="s">
+    <row r="21" spans="2:6">
+      <c r="D21" t="s">
         <v>1</v>
       </c>
       <c r="E21">
-        <v>4.52688691920903E-09</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6">
-      <c r="A22" s="1"/>
-      <c r="B22" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="2:6">
+      <c r="B22" t="s">
         <v>21</v>
       </c>
-      <c r="C22" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D22" s="1" t="s">
+      <c r="C22" t="s">
+        <v>26</v>
+      </c>
+      <c r="D22" t="s">
         <v>0</v>
       </c>
       <c r="F22">
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:6">
-      <c r="A23" s="1"/>
-      <c r="B23" s="1"/>
-      <c r="C23" s="1"/>
-      <c r="D23" s="1" t="s">
+    <row r="23" spans="2:6">
+      <c r="D23" t="s">
         <v>1</v>
       </c>
       <c r="E23">
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:6">
-      <c r="A24" s="1"/>
-      <c r="B24" s="1" t="s">
+    <row r="24" spans="2:6">
+      <c r="B24" t="s">
         <v>23</v>
       </c>
-      <c r="C24" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D24" s="1" t="s">
+      <c r="C24" t="s">
+        <v>26</v>
+      </c>
+      <c r="D24" t="s">
         <v>0</v>
       </c>
       <c r="F24">
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:6">
-      <c r="A25" s="1"/>
-      <c r="B25" s="1"/>
-      <c r="C25" s="1"/>
-      <c r="D25" s="1" t="s">
+    <row r="25" spans="2:6">
+      <c r="D25" t="s">
         <v>1</v>
       </c>
       <c r="E25">
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:6">
-      <c r="A26" s="1"/>
-      <c r="B26" s="1" t="s">
+    <row r="26" spans="2:6">
+      <c r="B26" t="s">
         <v>24</v>
       </c>
-      <c r="C26" s="1" t="s">
+      <c r="C26" t="s">
         <v>25</v>
       </c>
-      <c r="D26" s="1" t="s">
+      <c r="D26" t="s">
         <v>0</v>
       </c>
       <c r="F26">
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:6">
-      <c r="A27" s="1"/>
-      <c r="B27" s="1"/>
-      <c r="C27" s="1"/>
-      <c r="D27" s="1" t="s">
+    <row r="27" spans="2:6">
+      <c r="D27" t="s">
         <v>1</v>
       </c>
       <c r="E27">

</xml_diff>